<commit_message>
Lead FedEx pre-read with same origin×dest O2D actual compare
Adds Table A0: SoCal constrained origin by dest region, builds directs
vs does not — directs slower on O2D actual on every major destination.

Co-authored-by: et844p <et844p@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/directs/fedex_preread_directs_speed.xlsx
+++ b/output/directs/fedex_preread_directs_speed.xlsx
@@ -8,12 +8,13 @@
   </bookViews>
   <sheets>
     <sheet name="01_Bottom_Line" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="02_SoCal_Constrained_Periods" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="03_Similar_BAU_Cohort" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="04_SoCal_10w_Direct_vs_Local" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="05_WC_to_Midwest" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="06_Network_Buckets" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="07_Discussion_Position" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="02_Same_OD_O2D" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="02_SoCal_Constrained_Periods" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="03_Similar_BAU_Cohort" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="04_SoCal_10w_Direct_vs_Local" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="05_WC_to_Midwest" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="06_Network_Buckets" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="07_Discussion_Position" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -52,6 +53,14 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
   <fills count="3">
@@ -93,7 +102,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -111,6 +120,12 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -494,10 +509,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="35" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>FedEx is pushing Wayfair to push directs. We do not yet see the O2D actual speed benefits needed to justify that.</t>
+    <row r="2" ht="45" customHeight="1">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>Proof lens: same SoCal constrained origin × same dest region — builds directs vs does not. Speed metric = O2D actual. Directs are slower on every major dest (+0.2d to +0.5d; Midwest +0.43d).</t>
         </is>
       </c>
     </row>
@@ -594,9 +609,9 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A11:F11"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A11:F11"/>
-    <mergeCell ref="A16:F16"/>
     <mergeCell ref="A10:F10"/>
     <mergeCell ref="A14:F14"/>
     <mergeCell ref="A5:F5"/>
@@ -612,6 +627,369 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Table A0 — Same origin (SoCal constrained) × dest region</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Builds directs vs does not build directs. Pass = lower O2D actual for directs. Result: directs slower on every major dest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>Dest region</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>Directs vol</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>No-direct vol</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>O2D actual (directs)</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>O2D actual (no direct)</t>
+        </is>
+      </c>
+      <c r="F4" s="11" t="inlineStr">
+        <is>
+          <t>Δ O2D (direct − no direct)</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="inlineStr">
+        <is>
+          <t>Direct IFR</t>
+        </is>
+      </c>
+      <c r="H4" s="11" t="inlineStr">
+        <is>
+          <t>No-direct IFR</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="n">
+        <v>66812</v>
+      </c>
+      <c r="C5" s="12" t="n">
+        <v>225809</v>
+      </c>
+      <c r="D5" s="12" t="n">
+        <v>7.45</v>
+      </c>
+      <c r="E5" s="12" t="n">
+        <v>7.02</v>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>+0.43d</t>
+        </is>
+      </c>
+      <c r="G5" s="12" t="inlineStr">
+        <is>
+          <t>87.7%</t>
+        </is>
+      </c>
+      <c r="H5" s="12" t="inlineStr">
+        <is>
+          <t>89.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Southeast</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="n">
+        <v>51184</v>
+      </c>
+      <c r="C6" s="12" t="n">
+        <v>161941</v>
+      </c>
+      <c r="D6" s="12" t="n">
+        <v>7.31</v>
+      </c>
+      <c r="E6" s="12" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="F6" s="12" t="inlineStr">
+        <is>
+          <t>+0.32d</t>
+        </is>
+      </c>
+      <c r="G6" s="12" t="inlineStr">
+        <is>
+          <t>87.9%</t>
+        </is>
+      </c>
+      <c r="H6" s="12" t="inlineStr">
+        <is>
+          <t>89.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="n">
+        <v>39731</v>
+      </c>
+      <c r="C7" s="12" t="n">
+        <v>255142</v>
+      </c>
+      <c r="D7" s="12" t="n">
+        <v>4.64</v>
+      </c>
+      <c r="E7" s="12" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="F7" s="12" t="inlineStr">
+        <is>
+          <t>+0.53d</t>
+        </is>
+      </c>
+      <c r="G7" s="12" t="inlineStr">
+        <is>
+          <t>88.5%</t>
+        </is>
+      </c>
+      <c r="H7" s="12" t="inlineStr">
+        <is>
+          <t>90.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>South Central</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="n">
+        <v>36265</v>
+      </c>
+      <c r="C8" s="12" t="n">
+        <v>157978</v>
+      </c>
+      <c r="D8" s="12" t="n">
+        <v>5.29</v>
+      </c>
+      <c r="E8" s="12" t="n">
+        <v>5.11</v>
+      </c>
+      <c r="F8" s="12" t="inlineStr">
+        <is>
+          <t>+0.18d</t>
+        </is>
+      </c>
+      <c r="G8" s="12" t="inlineStr">
+        <is>
+          <t>88.4%</t>
+        </is>
+      </c>
+      <c r="H8" s="12" t="inlineStr">
+        <is>
+          <t>89.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Northeast</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="n">
+        <v>34888</v>
+      </c>
+      <c r="C9" s="12" t="n">
+        <v>129936</v>
+      </c>
+      <c r="D9" s="12" t="n">
+        <v>7.68</v>
+      </c>
+      <c r="E9" s="12" t="n">
+        <v>7.36</v>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>+0.33d</t>
+        </is>
+      </c>
+      <c r="G9" s="12" t="inlineStr">
+        <is>
+          <t>87.2%</t>
+        </is>
+      </c>
+      <c r="H9" s="12" t="inlineStr">
+        <is>
+          <t>89.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>Florida</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="n">
+        <v>34477</v>
+      </c>
+      <c r="C10" s="12" t="n">
+        <v>94226</v>
+      </c>
+      <c r="D10" s="12" t="n">
+        <v>7.43</v>
+      </c>
+      <c r="E10" s="12" t="n">
+        <v>7.12</v>
+      </c>
+      <c r="F10" s="12" t="inlineStr">
+        <is>
+          <t>+0.31d</t>
+        </is>
+      </c>
+      <c r="G10" s="12" t="inlineStr">
+        <is>
+          <t>87.8%</t>
+        </is>
+      </c>
+      <c r="H10" s="12" t="inlineStr">
+        <is>
+          <t>89.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>Mid-Atlantic</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="n">
+        <v>32380</v>
+      </c>
+      <c r="C11" s="12" t="n">
+        <v>78206</v>
+      </c>
+      <c r="D11" s="12" t="n">
+        <v>7.55</v>
+      </c>
+      <c r="E11" s="12" t="n">
+        <v>7.17</v>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>+0.38d</t>
+        </is>
+      </c>
+      <c r="G11" s="12" t="inlineStr">
+        <is>
+          <t>88.0%</t>
+        </is>
+      </c>
+      <c r="H11" s="12" t="inlineStr">
+        <is>
+          <t>89.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>West Coast</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="n">
+        <v>65201</v>
+      </c>
+      <c r="C12" s="12" t="n">
+        <v>576858</v>
+      </c>
+      <c r="D12" s="12" t="n">
+        <v>4.62</v>
+      </c>
+      <c r="E12" s="12" t="n">
+        <v>3.51</v>
+      </c>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>+1.11d</t>
+        </is>
+      </c>
+      <c r="G12" s="12" t="inlineStr">
+        <is>
+          <t>88.2%</t>
+        </is>
+      </c>
+      <c r="H12" s="12" t="inlineStr">
+        <is>
+          <t>90.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>Negative Δ would mean directs faster. All major dests are positive → directs slower on O2D actual.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A15:H15"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -974,7 +1352,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1346,7 +1724,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1497,7 +1875,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1672,7 +2050,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1862,7 +2240,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>